<commit_message>
Judge convergence on the restored epoch
EarlyStopping(start_from_epoch=30) restores the best weights from epoch 31 on,
but convergence_check.csv used the minimum over all epochs. Adds
convergence_check_restored_epoch.csv for each protocol and updates
Supplementary Data S1. Seven runs restored a different epoch; all verdicts hold.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Supplementary_Data_S1.xlsx
+++ b/Supplementary_Data_S1.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Per-seed result of the pre-registered convergence check. Source: */convergence_check.csv</t>
+          <t>Per-seed convergence check on the restored model (best weights from epoch 31 on). Source: */convergence_check_restored_epoch.csv</t>
         </is>
       </c>
     </row>
@@ -11962,13 +11962,13 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11984,37 +11984,37 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>epochs_run</t>
+          <t>epochs</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>best_epoch</t>
+          <t>min_epoch_all</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>best_val_loss</t>
+          <t>min_ratio_all</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>constant_val_loss</t>
+          <t>restored_epoch</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>restored_val</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>restored_ratio</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>converged</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>final_train_loss</t>
         </is>
       </c>
     </row>
@@ -12034,19 +12034,19 @@
         <v>31</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>11.52851295471191</v>
+        <v>0.399</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>28.90820503234863</v>
+        <v>31</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.3987972598717688</v>
-      </c>
-      <c r="H2" s="4" t="b">
+        <v>11.529</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="I2" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="3">
@@ -12065,19 +12065,19 @@
         <v>29</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>12.54674530029297</v>
+        <v>0.434</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>28.90820503234863</v>
+        <v>35</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.4340202128168459</v>
-      </c>
-      <c r="H3" s="4" t="b">
+        <v>12.703</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="I3" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="4">
@@ -12096,19 +12096,19 @@
         <v>32</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>15.23516750335693</v>
+        <v>0.527</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>28.90820503234863</v>
+        <v>32</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.5270187992062667</v>
-      </c>
-      <c r="H4" s="4" t="b">
+        <v>15.235</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="I4" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="5">
@@ -12127,19 +12127,19 @@
         <v>86</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>12.57099723815918</v>
+        <v>0.435</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>28.90820503234863</v>
+        <v>86</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.4348591420356982</v>
-      </c>
-      <c r="H5" s="4" t="b">
+        <v>12.571</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="I5" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -12158,19 +12158,19 @@
         <v>43</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>10.85485553741455</v>
+        <v>0.375</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>28.90820503234863</v>
+        <v>43</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.3754939307116383</v>
-      </c>
-      <c r="H6" s="4" t="b">
+        <v>10.855</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="I6" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="7">
@@ -12189,19 +12189,19 @@
         <v>71</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>11.07884979248047</v>
+        <v>0.381</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>29.08147048950195</v>
+        <v>71</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.3809590645177242</v>
-      </c>
-      <c r="H7" s="4" t="b">
+        <v>11.079</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="I7" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>10.1069507598877</v>
       </c>
     </row>
     <row r="8">
@@ -12220,19 +12220,19 @@
         <v>75</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>10.60379600524902</v>
+        <v>0.365</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>29.08147048950195</v>
+        <v>75</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.3646237905705924</v>
-      </c>
-      <c r="H8" s="4" t="b">
+        <v>10.604</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="I8" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>9.964648246765137</v>
       </c>
     </row>
     <row r="9">
@@ -12251,19 +12251,19 @@
         <v>45</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>13.31274032592773</v>
+        <v>0.458</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>29.08147048950195</v>
+        <v>45</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.4577739743502126</v>
-      </c>
-      <c r="H9" s="4" t="b">
+        <v>13.313</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0.458</v>
+      </c>
+      <c r="I9" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>11.54624080657959</v>
       </c>
     </row>
     <row r="10">
@@ -12282,19 +12282,19 @@
         <v>69</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>15.16658973693848</v>
+        <v>0.522</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>29.08147048950195</v>
+        <v>69</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.5215207306113845</v>
-      </c>
-      <c r="H10" s="4" t="b">
+        <v>15.167</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="I10" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>11.27593994140625</v>
       </c>
     </row>
     <row r="11">
@@ -12313,19 +12313,19 @@
         <v>38</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>11.27132701873779</v>
+        <v>0.388</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>29.08147048950195</v>
+        <v>38</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.3875776165722638</v>
-      </c>
-      <c r="H11" s="4" t="b">
+        <v>11.271</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="I11" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>11.5394926071167</v>
       </c>
     </row>
     <row r="12">
@@ -12344,19 +12344,19 @@
         <v>63</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>10.91294288635254</v>
+        <v>0.379</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>28.80680656433105</v>
+        <v>63</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.3788320951849304</v>
-      </c>
-      <c r="H12" s="4" t="b">
+        <v>10.913</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="I12" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="13">
@@ -12375,19 +12375,19 @@
         <v>55</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>12.03601741790772</v>
+        <v>0.418</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>28.80680656433105</v>
+        <v>55</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.4178185246264284</v>
-      </c>
-      <c r="H13" s="4" t="b">
+        <v>12.036</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="I13" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="14">
@@ -12406,19 +12406,19 @@
         <v>30</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>11.1314582824707</v>
+        <v>0.386</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>28.80680656433105</v>
+        <v>36</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.3864176425669415</v>
-      </c>
-      <c r="H14" s="4" t="b">
+        <v>11.147</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="I14" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="15">
@@ -12437,19 +12437,19 @@
         <v>36</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>11.41899967193604</v>
+        <v>0.396</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>28.80680656433105</v>
+        <v>36</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.3963993595206482</v>
-      </c>
-      <c r="H15" s="4" t="b">
+        <v>11.419</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="I15" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I15" s="4" t="n">
-        <v/>
       </c>
     </row>
     <row r="16">
@@ -12468,19 +12468,19 @@
         <v>27</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>11.88245677947998</v>
+        <v>0.412</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>28.80680656433105</v>
+        <v>34</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.4124878178684681</v>
-      </c>
-      <c r="H16" s="4" t="b">
+        <v>11.892</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0.413</v>
+      </c>
+      <c r="I16" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -12621,7 +12621,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>val pinball loss, patience 15, from epoch 30, best weights restored</t>
+          <t>val pinball loss; monitoring starts after epoch 30; patience 15; best weights from epoch 31 on restored</t>
         </is>
       </c>
     </row>
@@ -12633,7 +12633,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>best val loss &lt;= 0.60 x constant-quantile loss</t>
+          <t>restored model val loss &lt;= 0.60 x constant-quantile loss</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Supplementary Data S1: add Tables S1-S2 (per-engine diagnostics)
Table S1 holds the IID hard-engine diagnostics and Table S2 the persistent shift-sensitive engines. Both moved
out of the Part I manuscript to fit IJPHM's length guidance; Section 6.7 keeps their key numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Supplementary_Data_S1.xlsx
+++ b/Supplementary_Data_S1.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="IID split" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DS-A split" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DS-B split" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DS-B thresholds" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Convergence" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Protocol" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Shift preprocessing" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IID split" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DS-A split" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DS-B split" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DS-B thresholds" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Convergence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shift preprocessing" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1 IID hard engines" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2 persistent engines" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +42,12 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -67,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -75,6 +83,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,6 +562,440 @@
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>NASA C-MAPSS FD004 training file only (61,249 rows, 249 engines); RUL clipped at 125 cycles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Table S1 IID hard engines</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Per-engine diagnostics of the three IID engines below 80% Balanced coverage (Part I, Section 6.7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Table S2 persistent engines</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Per-engine diagnostics of the five engines below 80% Balanced coverage under both shifts (Part I, Section 6.7).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Table S2. Persistent shift-sensitive engines (below 80% Balanced Engine CQR coverage under both DS-A and DS-B, seed 42). RMSE, MAE and signed bias (pred − true) in cycles; mid-life coverage on windows with 40 &lt; RUL ≤ 80. The dominant endpoint regime is the most frequent regime among the engine's test endpoints, with its share; all DS-A endpoints are Regime 0 by construction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Signed bias</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Balanced cov. (%)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Mid-life cov. (%)</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Dominant endpoint regime</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DS-A</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D4" t="n">
+        <v>51.86</v>
+      </c>
+      <c r="E4" t="n">
+        <v>45.23</v>
+      </c>
+      <c r="F4" t="n">
+        <v>45.23</v>
+      </c>
+      <c r="G4" t="n">
+        <v>48</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0 (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DS-B</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>23</v>
+      </c>
+      <c r="D5" t="n">
+        <v>49.41</v>
+      </c>
+      <c r="E5" t="n">
+        <v>41.46</v>
+      </c>
+      <c r="F5" t="n">
+        <v>41.46</v>
+      </c>
+      <c r="G5" t="n">
+        <v>60.87</v>
+      </c>
+      <c r="H5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>4 (26%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>156</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DS-A</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="E6" t="n">
+        <v>44.86</v>
+      </c>
+      <c r="F6" t="n">
+        <v>44.86</v>
+      </c>
+      <c r="G6" t="n">
+        <v>57.69</v>
+      </c>
+      <c r="H6" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0 (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>156</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DS-B</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" t="n">
+        <v>44</v>
+      </c>
+      <c r="G7" t="n">
+        <v>55</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1 (35%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>184</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DS-A</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>79</v>
+      </c>
+      <c r="D8" t="n">
+        <v>37.36</v>
+      </c>
+      <c r="E8" t="n">
+        <v>26.48</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-26.28</v>
+      </c>
+      <c r="G8" t="n">
+        <v>67.09</v>
+      </c>
+      <c r="H8" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0 (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>184</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DS-B</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>73</v>
+      </c>
+      <c r="D9" t="n">
+        <v>39.95</v>
+      </c>
+      <c r="E9" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-27.03</v>
+      </c>
+      <c r="G9" t="n">
+        <v>63.01</v>
+      </c>
+      <c r="H9" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0 (30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>194</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DS-A</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>29</v>
+      </c>
+      <c r="D10" t="n">
+        <v>32.32</v>
+      </c>
+      <c r="E10" t="n">
+        <v>26.84</v>
+      </c>
+      <c r="F10" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="G10" t="n">
+        <v>75.86</v>
+      </c>
+      <c r="H10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0 (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>194</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DS-B</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>33</v>
+      </c>
+      <c r="D11" t="n">
+        <v>33.59</v>
+      </c>
+      <c r="E11" t="n">
+        <v>25.97</v>
+      </c>
+      <c r="F11" t="n">
+        <v>25.77</v>
+      </c>
+      <c r="G11" t="n">
+        <v>78.79000000000001</v>
+      </c>
+      <c r="H11" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0 (27%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>240</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DS-A</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>32</v>
+      </c>
+      <c r="D12" t="n">
+        <v>42.97</v>
+      </c>
+      <c r="E12" t="n">
+        <v>36.27</v>
+      </c>
+      <c r="F12" t="n">
+        <v>36.27</v>
+      </c>
+      <c r="G12" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>30</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0 (all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>240</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DS-B</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>16</v>
+      </c>
+      <c r="D13" t="n">
+        <v>50.91</v>
+      </c>
+      <c r="E13" t="n">
+        <v>45.75</v>
+      </c>
+      <c r="F13" t="n">
+        <v>45.75</v>
+      </c>
+      <c r="G13" t="n">
+        <v>50</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>4 (25%)</t>
         </is>
       </c>
     </row>
@@ -12904,4 +13348,171 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Table S1. Standard (IID) hard-engine diagnostics (seed 42): engines below 80% Balanced Engine CQR coverage. RMSE, MAE and mean bias (pred − true) in cycles; misses are the share of windows below the lower or above the upper bound; mid-life coverage on windows with 40 &lt; RUL ≤ 80.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Mean bias (pred − true)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Balanced PICP (%)</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Below-lower miss (%)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Above-upper miss (%)</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Mid-life cov. (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B4" t="n">
+        <v>350</v>
+      </c>
+      <c r="C4" t="n">
+        <v>35.87</v>
+      </c>
+      <c r="D4" t="n">
+        <v>24.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-24</v>
+      </c>
+      <c r="F4" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>28.57</v>
+      </c>
+      <c r="I4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B5" t="n">
+        <v>230</v>
+      </c>
+      <c r="C5" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19.67</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-10.09</v>
+      </c>
+      <c r="F5" t="n">
+        <v>79.56999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="H5" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="I5" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B6" t="n">
+        <v>182</v>
+      </c>
+      <c r="C6" t="n">
+        <v>37.98</v>
+      </c>
+      <c r="D6" t="n">
+        <v>26.48</v>
+      </c>
+      <c r="E6" t="n">
+        <v>26.45</v>
+      </c>
+      <c r="F6" t="n">
+        <v>72.53</v>
+      </c>
+      <c r="G6" t="n">
+        <v>27.47</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Use FD004 unit numbers for the IID engines
The saved IID files number engines by position (fit and internal_val 1-200 among the sorted
training units, calibration and evaluation 1-49 among the sorted validation units), while the
DS-A and DS-B files use FD004 unit numbers. IID engine 36 is therefore unit 184, the same engine
as the persistent shift engine 184.

- iid_engine_to_unit.csv: unit of every IID engine; reproduces the window counts of all four
  splits (34,983 / 8,713 / 4,909 / 5,423) and each evaluation engine's failure cycle.
- Supplementary_Data_S1.xlsx: Table S1 lists units 184, 185, 247 (saved-file numbers 36, 37, 49
  in a new last column); the IID split sheet gains a unit_id column.
- README: explains the numbering.

Result folders and their SHA-256 manifests are unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Supplementary_Data_S1.xlsx
+++ b/Supplementary_Data_S1.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -586,6 +586,18 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>Per-engine diagnostics of the five engines below 80% Balanced coverage under both shifts (Part I, Section 6.7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IID engine numbering</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The saved IID files number engines by position: fit and internal_val (1-200) among the sorted training units, calibration and evaluation (1-49) among the sorted validation units. Sheet 'IID split' gives the FD004 unit_id of every engine; Table S1 is by unit.</t>
         </is>
       </c>
     </row>
@@ -621,7 +633,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -1010,12 +1021,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C250"/>
+  <dimension ref="A1:D250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1031,7 +1042,12 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>engine_index</t>
+          <t>position_in_saved_files</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>unit_id</t>
         </is>
       </c>
     </row>
@@ -1049,6 +1065,9 @@
       <c r="C2" s="4" t="n">
         <v>80</v>
       </c>
+      <c r="D2" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1064,6 +1083,9 @@
       <c r="C3" s="4" t="n">
         <v>198</v>
       </c>
+      <c r="D3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1079,6 +1101,9 @@
       <c r="C4" s="4" t="n">
         <v>39</v>
       </c>
+      <c r="D4" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1094,6 +1119,9 @@
       <c r="C5" s="4" t="n">
         <v>25</v>
       </c>
+      <c r="D5" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1109,6 +1137,9 @@
       <c r="C6" s="4" t="n">
         <v>123</v>
       </c>
+      <c r="D6" t="n">
+        <v>151</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1124,6 +1155,9 @@
       <c r="C7" s="4" t="n">
         <v>196</v>
       </c>
+      <c r="D7" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1139,6 +1173,9 @@
       <c r="C8" s="4" t="n">
         <v>30</v>
       </c>
+      <c r="D8" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1154,6 +1191,9 @@
       <c r="C9" s="4" t="n">
         <v>20</v>
       </c>
+      <c r="D9" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1169,6 +1209,9 @@
       <c r="C10" s="4" t="n">
         <v>144</v>
       </c>
+      <c r="D10" t="n">
+        <v>178</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1184,6 +1227,9 @@
       <c r="C11" s="4" t="n">
         <v>87</v>
       </c>
+      <c r="D11" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1199,6 +1245,9 @@
       <c r="C12" s="4" t="n">
         <v>115</v>
       </c>
+      <c r="D12" t="n">
+        <v>143</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1214,6 +1263,9 @@
       <c r="C13" s="4" t="n">
         <v>174</v>
       </c>
+      <c r="D13" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1229,6 +1281,9 @@
       <c r="C14" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1244,6 +1299,9 @@
       <c r="C15" s="4" t="n">
         <v>127</v>
       </c>
+      <c r="D15" t="n">
+        <v>155</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1259,6 +1317,9 @@
       <c r="C16" s="4" t="n">
         <v>118</v>
       </c>
+      <c r="D16" t="n">
+        <v>146</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1274,6 +1335,9 @@
       <c r="C17" s="4" t="n">
         <v>74</v>
       </c>
+      <c r="D17" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1289,6 +1353,9 @@
       <c r="C18" s="4" t="n">
         <v>141</v>
       </c>
+      <c r="D18" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1304,6 +1371,9 @@
       <c r="C19" s="4" t="n">
         <v>99</v>
       </c>
+      <c r="D19" t="n">
+        <v>125</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1319,6 +1389,9 @@
       <c r="C20" s="4" t="n">
         <v>173</v>
       </c>
+      <c r="D20" t="n">
+        <v>219</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1334,6 +1407,9 @@
       <c r="C21" s="4" t="n">
         <v>97</v>
       </c>
+      <c r="D21" t="n">
+        <v>123</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1349,6 +1425,9 @@
       <c r="C22" s="4" t="n">
         <v>170</v>
       </c>
+      <c r="D22" t="n">
+        <v>215</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1364,6 +1443,9 @@
       <c r="C23" s="4" t="n">
         <v>98</v>
       </c>
+      <c r="D23" t="n">
+        <v>124</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1379,6 +1461,9 @@
       <c r="C24" s="4" t="n">
         <v>32</v>
       </c>
+      <c r="D24" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1394,6 +1479,9 @@
       <c r="C25" s="4" t="n">
         <v>13</v>
       </c>
+      <c r="D25" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1409,6 +1497,9 @@
       <c r="C26" s="4" t="n">
         <v>36</v>
       </c>
+      <c r="D26" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1424,6 +1515,9 @@
       <c r="C27" s="4" t="n">
         <v>120</v>
       </c>
+      <c r="D27" t="n">
+        <v>148</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1439,6 +1533,9 @@
       <c r="C28" s="4" t="n">
         <v>43</v>
       </c>
+      <c r="D28" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1454,6 +1551,9 @@
       <c r="C29" s="4" t="n">
         <v>190</v>
       </c>
+      <c r="D29" t="n">
+        <v>237</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1469,6 +1569,9 @@
       <c r="C30" s="4" t="n">
         <v>91</v>
       </c>
+      <c r="D30" t="n">
+        <v>114</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1484,6 +1587,9 @@
       <c r="C31" s="4" t="n">
         <v>137</v>
       </c>
+      <c r="D31" t="n">
+        <v>168</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1499,6 +1605,9 @@
       <c r="C32" s="4" t="n">
         <v>52</v>
       </c>
+      <c r="D32" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1514,6 +1623,9 @@
       <c r="C33" s="4" t="n">
         <v>128</v>
       </c>
+      <c r="D33" t="n">
+        <v>156</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1529,6 +1641,9 @@
       <c r="C34" s="4" t="n">
         <v>163</v>
       </c>
+      <c r="D34" t="n">
+        <v>208</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1544,6 +1659,9 @@
       <c r="C35" s="4" t="n">
         <v>42</v>
       </c>
+      <c r="D35" t="n">
+        <v>54</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1559,6 +1677,9 @@
       <c r="C36" s="4" t="n">
         <v>119</v>
       </c>
+      <c r="D36" t="n">
+        <v>147</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -1574,6 +1695,9 @@
       <c r="C37" s="4" t="n">
         <v>114</v>
       </c>
+      <c r="D37" t="n">
+        <v>142</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -1589,6 +1713,9 @@
       <c r="C38" s="4" t="n">
         <v>27</v>
       </c>
+      <c r="D38" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -1604,6 +1731,9 @@
       <c r="C39" s="4" t="n">
         <v>140</v>
       </c>
+      <c r="D39" t="n">
+        <v>171</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1619,6 +1749,9 @@
       <c r="C40" s="4" t="n">
         <v>101</v>
       </c>
+      <c r="D40" t="n">
+        <v>127</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -1634,6 +1767,9 @@
       <c r="C41" s="4" t="n">
         <v>112</v>
       </c>
+      <c r="D41" t="n">
+        <v>139</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -1649,6 +1785,9 @@
       <c r="C42" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="D42" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -1664,6 +1803,9 @@
       <c r="C43" s="4" t="n">
         <v>78</v>
       </c>
+      <c r="D43" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -1679,6 +1821,9 @@
       <c r="C44" s="4" t="n">
         <v>47</v>
       </c>
+      <c r="D44" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -1694,6 +1839,9 @@
       <c r="C45" s="4" t="n">
         <v>188</v>
       </c>
+      <c r="D45" t="n">
+        <v>235</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -1709,6 +1857,9 @@
       <c r="C46" s="4" t="n">
         <v>192</v>
       </c>
+      <c r="D46" t="n">
+        <v>239</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -1724,6 +1875,9 @@
       <c r="C47" s="4" t="n">
         <v>86</v>
       </c>
+      <c r="D47" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -1739,6 +1893,9 @@
       <c r="C48" s="4" t="n">
         <v>162</v>
       </c>
+      <c r="D48" t="n">
+        <v>207</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -1754,6 +1911,9 @@
       <c r="C49" s="4" t="n">
         <v>37</v>
       </c>
+      <c r="D49" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -1769,6 +1929,9 @@
       <c r="C50" s="4" t="n">
         <v>191</v>
       </c>
+      <c r="D50" t="n">
+        <v>238</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -1784,6 +1947,9 @@
       <c r="C51" s="4" t="n">
         <v>62</v>
       </c>
+      <c r="D51" t="n">
+        <v>79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -1799,6 +1965,9 @@
       <c r="C52" s="4" t="n">
         <v>23</v>
       </c>
+      <c r="D52" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -1814,6 +1983,9 @@
       <c r="C53" s="4" t="n">
         <v>142</v>
       </c>
+      <c r="D53" t="n">
+        <v>175</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -1829,6 +2001,9 @@
       <c r="C54" s="4" t="n">
         <v>102</v>
       </c>
+      <c r="D54" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -1844,6 +2019,9 @@
       <c r="C55" s="4" t="n">
         <v>34</v>
       </c>
+      <c r="D55" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -1859,6 +2037,9 @@
       <c r="C56" s="4" t="n">
         <v>12</v>
       </c>
+      <c r="D56" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -1874,6 +2055,9 @@
       <c r="C57" s="4" t="n">
         <v>195</v>
       </c>
+      <c r="D57" t="n">
+        <v>243</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -1889,6 +2073,9 @@
       <c r="C58" s="4" t="n">
         <v>160</v>
       </c>
+      <c r="D58" t="n">
+        <v>205</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -1904,6 +2091,9 @@
       <c r="C59" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="D59" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -1919,6 +2109,9 @@
       <c r="C60" s="4" t="n">
         <v>28</v>
       </c>
+      <c r="D60" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -1934,6 +2127,9 @@
       <c r="C61" s="4" t="n">
         <v>121</v>
       </c>
+      <c r="D61" t="n">
+        <v>149</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -1949,6 +2145,9 @@
       <c r="C62" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="D62" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -1964,6 +2163,9 @@
       <c r="C63" s="4" t="n">
         <v>33</v>
       </c>
+      <c r="D63" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -1979,6 +2181,9 @@
       <c r="C64" s="4" t="n">
         <v>143</v>
       </c>
+      <c r="D64" t="n">
+        <v>177</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -1994,6 +2199,9 @@
       <c r="C65" s="4" t="n">
         <v>146</v>
       </c>
+      <c r="D65" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -2009,6 +2217,9 @@
       <c r="C66" s="4" t="n">
         <v>110</v>
       </c>
+      <c r="D66" t="n">
+        <v>136</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -2024,6 +2235,9 @@
       <c r="C67" s="4" t="n">
         <v>145</v>
       </c>
+      <c r="D67" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -2039,6 +2253,9 @@
       <c r="C68" s="4" t="n">
         <v>11</v>
       </c>
+      <c r="D68" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -2054,6 +2271,9 @@
       <c r="C69" s="4" t="n">
         <v>63</v>
       </c>
+      <c r="D69" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -2069,6 +2289,9 @@
       <c r="C70" s="4" t="n">
         <v>113</v>
       </c>
+      <c r="D70" t="n">
+        <v>140</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -2084,6 +2307,9 @@
       <c r="C71" s="4" t="n">
         <v>147</v>
       </c>
+      <c r="D71" t="n">
+        <v>182</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -2099,6 +2325,9 @@
       <c r="C72" s="4" t="n">
         <v>167</v>
       </c>
+      <c r="D72" t="n">
+        <v>212</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -2114,6 +2343,9 @@
       <c r="C73" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -2129,6 +2361,9 @@
       <c r="C74" s="4" t="n">
         <v>199</v>
       </c>
+      <c r="D74" t="n">
+        <v>248</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -2144,6 +2379,9 @@
       <c r="C75" s="4" t="n">
         <v>154</v>
       </c>
+      <c r="D75" t="n">
+        <v>192</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -2159,6 +2397,9 @@
       <c r="C76" s="4" t="n">
         <v>71</v>
       </c>
+      <c r="D76" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -2174,6 +2415,9 @@
       <c r="C77" s="4" t="n">
         <v>124</v>
       </c>
+      <c r="D77" t="n">
+        <v>152</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -2189,6 +2433,9 @@
       <c r="C78" s="4" t="n">
         <v>65</v>
       </c>
+      <c r="D78" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -2204,6 +2451,9 @@
       <c r="C79" s="4" t="n">
         <v>45</v>
       </c>
+      <c r="D79" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -2219,6 +2469,9 @@
       <c r="C80" s="4" t="n">
         <v>164</v>
       </c>
+      <c r="D80" t="n">
+        <v>209</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -2234,6 +2487,9 @@
       <c r="C81" s="4" t="n">
         <v>29</v>
       </c>
+      <c r="D81" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -2249,6 +2505,9 @@
       <c r="C82" s="4" t="n">
         <v>41</v>
       </c>
+      <c r="D82" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -2264,6 +2523,9 @@
       <c r="C83" s="4" t="n">
         <v>109</v>
       </c>
+      <c r="D83" t="n">
+        <v>135</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -2279,6 +2541,9 @@
       <c r="C84" s="4" t="n">
         <v>156</v>
       </c>
+      <c r="D84" t="n">
+        <v>198</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -2294,6 +2559,9 @@
       <c r="C85" s="4" t="n">
         <v>157</v>
       </c>
+      <c r="D85" t="n">
+        <v>199</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -2309,6 +2577,9 @@
       <c r="C86" s="4" t="n">
         <v>26</v>
       </c>
+      <c r="D86" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -2324,6 +2595,9 @@
       <c r="C87" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="D87" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -2339,6 +2613,9 @@
       <c r="C88" s="4" t="n">
         <v>185</v>
       </c>
+      <c r="D88" t="n">
+        <v>232</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -2354,6 +2631,9 @@
       <c r="C89" s="4" t="n">
         <v>148</v>
       </c>
+      <c r="D89" t="n">
+        <v>183</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -2369,6 +2649,9 @@
       <c r="C90" s="4" t="n">
         <v>82</v>
       </c>
+      <c r="D90" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -2384,6 +2667,9 @@
       <c r="C91" s="4" t="n">
         <v>40</v>
       </c>
+      <c r="D91" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -2399,6 +2685,9 @@
       <c r="C92" s="4" t="n">
         <v>169</v>
       </c>
+      <c r="D92" t="n">
+        <v>214</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -2414,6 +2703,9 @@
       <c r="C93" s="4" t="n">
         <v>48</v>
       </c>
+      <c r="D93" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -2429,6 +2721,9 @@
       <c r="C94" s="4" t="n">
         <v>95</v>
       </c>
+      <c r="D94" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -2444,6 +2739,9 @@
       <c r="C95" s="4" t="n">
         <v>155</v>
       </c>
+      <c r="D95" t="n">
+        <v>193</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -2459,6 +2757,9 @@
       <c r="C96" s="4" t="n">
         <v>44</v>
       </c>
+      <c r="D96" t="n">
+        <v>57</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -2474,6 +2775,9 @@
       <c r="C97" s="4" t="n">
         <v>139</v>
       </c>
+      <c r="D97" t="n">
+        <v>170</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -2489,6 +2793,9 @@
       <c r="C98" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="D98" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -2504,6 +2811,9 @@
       <c r="C99" s="4" t="n">
         <v>106</v>
       </c>
+      <c r="D99" t="n">
+        <v>132</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -2519,6 +2829,9 @@
       <c r="C100" s="4" t="n">
         <v>54</v>
       </c>
+      <c r="D100" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -2534,6 +2847,9 @@
       <c r="C101" s="4" t="n">
         <v>134</v>
       </c>
+      <c r="D101" t="n">
+        <v>165</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -2549,6 +2865,9 @@
       <c r="C102" s="4" t="n">
         <v>181</v>
       </c>
+      <c r="D102" t="n">
+        <v>228</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -2564,6 +2883,9 @@
       <c r="C103" s="4" t="n">
         <v>179</v>
       </c>
+      <c r="D103" t="n">
+        <v>226</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -2579,6 +2901,9 @@
       <c r="C104" s="4" t="n">
         <v>186</v>
       </c>
+      <c r="D104" t="n">
+        <v>233</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -2594,6 +2919,9 @@
       <c r="C105" s="4" t="n">
         <v>50</v>
       </c>
+      <c r="D105" t="n">
+        <v>64</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -2609,6 +2937,9 @@
       <c r="C106" s="4" t="n">
         <v>81</v>
       </c>
+      <c r="D106" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -2624,6 +2955,9 @@
       <c r="C107" s="4" t="n">
         <v>35</v>
       </c>
+      <c r="D107" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -2639,6 +2973,9 @@
       <c r="C108" s="4" t="n">
         <v>8</v>
       </c>
+      <c r="D108" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -2654,6 +2991,9 @@
       <c r="C109" s="4" t="n">
         <v>111</v>
       </c>
+      <c r="D109" t="n">
+        <v>137</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -2669,6 +3009,9 @@
       <c r="C110" s="4" t="n">
         <v>92</v>
       </c>
+      <c r="D110" t="n">
+        <v>116</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -2684,6 +3027,9 @@
       <c r="C111" s="4" t="n">
         <v>84</v>
       </c>
+      <c r="D111" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -2699,6 +3045,9 @@
       <c r="C112" s="4" t="n">
         <v>177</v>
       </c>
+      <c r="D112" t="n">
+        <v>223</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -2714,6 +3063,9 @@
       <c r="C113" s="4" t="n">
         <v>182</v>
       </c>
+      <c r="D113" t="n">
+        <v>229</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -2729,6 +3081,9 @@
       <c r="C114" s="4" t="n">
         <v>90</v>
       </c>
+      <c r="D114" t="n">
+        <v>111</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -2744,6 +3099,9 @@
       <c r="C115" s="4" t="n">
         <v>9</v>
       </c>
+      <c r="D115" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -2759,6 +3117,9 @@
       <c r="C116" s="4" t="n">
         <v>14</v>
       </c>
+      <c r="D116" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -2774,6 +3135,9 @@
       <c r="C117" s="4" t="n">
         <v>60</v>
       </c>
+      <c r="D117" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -2789,6 +3153,9 @@
       <c r="C118" s="4" t="n">
         <v>172</v>
       </c>
+      <c r="D118" t="n">
+        <v>218</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -2804,6 +3171,9 @@
       <c r="C119" s="4" t="n">
         <v>132</v>
       </c>
+      <c r="D119" t="n">
+        <v>162</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -2819,6 +3189,9 @@
       <c r="C120" s="4" t="n">
         <v>18</v>
       </c>
+      <c r="D120" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -2834,6 +3207,9 @@
       <c r="C121" s="4" t="n">
         <v>73</v>
       </c>
+      <c r="D121" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -2849,6 +3225,9 @@
       <c r="C122" s="4" t="n">
         <v>176</v>
       </c>
+      <c r="D122" t="n">
+        <v>222</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -2864,6 +3243,9 @@
       <c r="C123" s="4" t="n">
         <v>135</v>
       </c>
+      <c r="D123" t="n">
+        <v>166</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -2879,6 +3261,9 @@
       <c r="C124" s="4" t="n">
         <v>168</v>
       </c>
+      <c r="D124" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -2894,6 +3279,9 @@
       <c r="C125" s="4" t="n">
         <v>184</v>
       </c>
+      <c r="D125" t="n">
+        <v>231</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -2909,6 +3297,9 @@
       <c r="C126" s="4" t="n">
         <v>64</v>
       </c>
+      <c r="D126" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -2924,6 +3315,9 @@
       <c r="C127" s="4" t="n">
         <v>55</v>
       </c>
+      <c r="D127" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -2939,6 +3333,9 @@
       <c r="C128" s="4" t="n">
         <v>108</v>
       </c>
+      <c r="D128" t="n">
+        <v>134</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -2954,6 +3351,9 @@
       <c r="C129" s="4" t="n">
         <v>51</v>
       </c>
+      <c r="D129" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
@@ -2969,6 +3369,9 @@
       <c r="C130" s="4" t="n">
         <v>197</v>
       </c>
+      <c r="D130" t="n">
+        <v>245</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -2984,6 +3387,9 @@
       <c r="C131" s="4" t="n">
         <v>59</v>
       </c>
+      <c r="D131" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -2999,6 +3405,9 @@
       <c r="C132" s="4" t="n">
         <v>49</v>
       </c>
+      <c r="D132" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -3014,6 +3423,9 @@
       <c r="C133" s="4" t="n">
         <v>89</v>
       </c>
+      <c r="D133" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -3029,6 +3441,9 @@
       <c r="C134" s="4" t="n">
         <v>22</v>
       </c>
+      <c r="D134" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -3044,6 +3459,9 @@
       <c r="C135" s="4" t="n">
         <v>58</v>
       </c>
+      <c r="D135" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -3059,6 +3477,9 @@
       <c r="C136" s="4" t="n">
         <v>161</v>
       </c>
+      <c r="D136" t="n">
+        <v>206</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -3074,6 +3495,9 @@
       <c r="C137" s="4" t="n">
         <v>193</v>
       </c>
+      <c r="D137" t="n">
+        <v>241</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -3089,6 +3513,9 @@
       <c r="C138" s="4" t="n">
         <v>130</v>
       </c>
+      <c r="D138" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -3104,6 +3531,9 @@
       <c r="C139" s="4" t="n">
         <v>38</v>
       </c>
+      <c r="D139" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -3119,6 +3549,9 @@
       <c r="C140" s="4" t="n">
         <v>158</v>
       </c>
+      <c r="D140" t="n">
+        <v>203</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -3134,6 +3567,9 @@
       <c r="C141" s="4" t="n">
         <v>194</v>
       </c>
+      <c r="D141" t="n">
+        <v>242</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -3149,6 +3585,9 @@
       <c r="C142" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="D142" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -3164,6 +3603,9 @@
       <c r="C143" s="4" t="n">
         <v>53</v>
       </c>
+      <c r="D143" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -3179,6 +3621,9 @@
       <c r="C144" s="4" t="n">
         <v>150</v>
       </c>
+      <c r="D144" t="n">
+        <v>187</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -3194,6 +3639,9 @@
       <c r="C145" s="4" t="n">
         <v>131</v>
       </c>
+      <c r="D145" t="n">
+        <v>161</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -3209,6 +3657,9 @@
       <c r="C146" s="4" t="n">
         <v>152</v>
       </c>
+      <c r="D146" t="n">
+        <v>189</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -3224,6 +3675,9 @@
       <c r="C147" s="4" t="n">
         <v>104</v>
       </c>
+      <c r="D147" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -3239,6 +3693,9 @@
       <c r="C148" s="4" t="n">
         <v>100</v>
       </c>
+      <c r="D148" t="n">
+        <v>126</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -3254,6 +3711,9 @@
       <c r="C149" s="4" t="n">
         <v>117</v>
       </c>
+      <c r="D149" t="n">
+        <v>145</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -3269,6 +3729,9 @@
       <c r="C150" s="4" t="n">
         <v>88</v>
       </c>
+      <c r="D150" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -3284,6 +3747,9 @@
       <c r="C151" s="4" t="n">
         <v>75</v>
       </c>
+      <c r="D151" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -3299,6 +3765,9 @@
       <c r="C152" s="4" t="n">
         <v>122</v>
       </c>
+      <c r="D152" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -3314,6 +3783,9 @@
       <c r="C153" s="4" t="n">
         <v>200</v>
       </c>
+      <c r="D153" t="n">
+        <v>249</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -3329,6 +3801,9 @@
       <c r="C154" s="4" t="n">
         <v>21</v>
       </c>
+      <c r="D154" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -3344,6 +3819,9 @@
       <c r="C155" s="4" t="n">
         <v>189</v>
       </c>
+      <c r="D155" t="n">
+        <v>236</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -3359,6 +3837,9 @@
       <c r="C156" s="4" t="n">
         <v>72</v>
       </c>
+      <c r="D156" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -3374,6 +3855,9 @@
       <c r="C157" s="4" t="n">
         <v>107</v>
       </c>
+      <c r="D157" t="n">
+        <v>133</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -3389,6 +3873,9 @@
       <c r="C158" s="4" t="n">
         <v>15</v>
       </c>
+      <c r="D158" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -3404,6 +3891,9 @@
       <c r="C159" s="4" t="n">
         <v>93</v>
       </c>
+      <c r="D159" t="n">
+        <v>117</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -3419,6 +3909,9 @@
       <c r="C160" s="4" t="n">
         <v>180</v>
       </c>
+      <c r="D160" t="n">
+        <v>227</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -3434,6 +3927,9 @@
       <c r="C161" s="4" t="n">
         <v>103</v>
       </c>
+      <c r="D161" t="n">
+        <v>129</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -3449,6 +3945,9 @@
       <c r="C162" s="4" t="n">
         <v>96</v>
       </c>
+      <c r="D162" t="n">
+        <v>122</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -3464,6 +3963,9 @@
       <c r="C163" s="4" t="n">
         <v>16</v>
       </c>
+      <c r="D163" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -3479,6 +3981,9 @@
       <c r="C164" s="4" t="n">
         <v>31</v>
       </c>
+      <c r="D164" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -3494,6 +3999,9 @@
       <c r="C165" s="4" t="n">
         <v>159</v>
       </c>
+      <c r="D165" t="n">
+        <v>204</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -3509,6 +4017,9 @@
       <c r="C166" s="4" t="n">
         <v>129</v>
       </c>
+      <c r="D166" t="n">
+        <v>157</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -3524,6 +4035,9 @@
       <c r="C167" s="4" t="n">
         <v>116</v>
       </c>
+      <c r="D167" t="n">
+        <v>144</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -3539,6 +4053,9 @@
       <c r="C168" s="4" t="n">
         <v>70</v>
       </c>
+      <c r="D168" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -3554,6 +4071,9 @@
       <c r="C169" s="4" t="n">
         <v>171</v>
       </c>
+      <c r="D169" t="n">
+        <v>217</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -3569,6 +4089,9 @@
       <c r="C170" s="4" t="n">
         <v>175</v>
       </c>
+      <c r="D170" t="n">
+        <v>221</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -3584,6 +4107,9 @@
       <c r="C171" s="4" t="n">
         <v>46</v>
       </c>
+      <c r="D171" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -3599,6 +4125,9 @@
       <c r="C172" s="4" t="n">
         <v>67</v>
       </c>
+      <c r="D172" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -3614,6 +4143,9 @@
       <c r="C173" s="4" t="n">
         <v>183</v>
       </c>
+      <c r="D173" t="n">
+        <v>230</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -3629,6 +4161,9 @@
       <c r="C174" s="4" t="n">
         <v>166</v>
       </c>
+      <c r="D174" t="n">
+        <v>211</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -3644,6 +4179,9 @@
       <c r="C175" s="4" t="n">
         <v>79</v>
       </c>
+      <c r="D175" t="n">
+        <v>96</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -3659,6 +4197,9 @@
       <c r="C176" s="4" t="n">
         <v>187</v>
       </c>
+      <c r="D176" t="n">
+        <v>234</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -3674,6 +4215,9 @@
       <c r="C177" s="4" t="n">
         <v>178</v>
       </c>
+      <c r="D177" t="n">
+        <v>225</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -3689,6 +4233,9 @@
       <c r="C178" s="4" t="n">
         <v>57</v>
       </c>
+      <c r="D178" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -3704,6 +4251,9 @@
       <c r="C179" s="4" t="n">
         <v>153</v>
       </c>
+      <c r="D179" t="n">
+        <v>190</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -3719,6 +4269,9 @@
       <c r="C180" s="4" t="n">
         <v>83</v>
       </c>
+      <c r="D180" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -3734,6 +4287,9 @@
       <c r="C181" s="4" t="n">
         <v>69</v>
       </c>
+      <c r="D181" t="n">
+        <v>86</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -3749,6 +4305,9 @@
       <c r="C182" s="4" t="n">
         <v>125</v>
       </c>
+      <c r="D182" t="n">
+        <v>153</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -3764,6 +4323,9 @@
       <c r="C183" s="4" t="n">
         <v>17</v>
       </c>
+      <c r="D183" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -3779,6 +4341,9 @@
       <c r="C184" s="4" t="n">
         <v>149</v>
       </c>
+      <c r="D184" t="n">
+        <v>186</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -3794,6 +4359,9 @@
       <c r="C185" s="4" t="n">
         <v>94</v>
       </c>
+      <c r="D185" t="n">
+        <v>118</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -3809,6 +4377,9 @@
       <c r="C186" s="4" t="n">
         <v>66</v>
       </c>
+      <c r="D186" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -3824,6 +4395,9 @@
       <c r="C187" s="4" t="n">
         <v>61</v>
       </c>
+      <c r="D187" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
@@ -3839,6 +4413,9 @@
       <c r="C188" s="4" t="n">
         <v>85</v>
       </c>
+      <c r="D188" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -3854,6 +4431,9 @@
       <c r="C189" s="4" t="n">
         <v>68</v>
       </c>
+      <c r="D189" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -3869,6 +4449,9 @@
       <c r="C190" s="4" t="n">
         <v>126</v>
       </c>
+      <c r="D190" t="n">
+        <v>154</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -3884,6 +4467,9 @@
       <c r="C191" s="4" t="n">
         <v>133</v>
       </c>
+      <c r="D191" t="n">
+        <v>164</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -3899,6 +4485,9 @@
       <c r="C192" s="4" t="n">
         <v>10</v>
       </c>
+      <c r="D192" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
@@ -3914,6 +4503,9 @@
       <c r="C193" s="4" t="n">
         <v>19</v>
       </c>
+      <c r="D193" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
@@ -3929,6 +4521,9 @@
       <c r="C194" s="4" t="n">
         <v>56</v>
       </c>
+      <c r="D194" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
@@ -3944,6 +4539,9 @@
       <c r="C195" s="4" t="n">
         <v>76</v>
       </c>
+      <c r="D195" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -3959,6 +4557,9 @@
       <c r="C196" s="4" t="n">
         <v>151</v>
       </c>
+      <c r="D196" t="n">
+        <v>188</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -3974,6 +4575,9 @@
       <c r="C197" s="4" t="n">
         <v>105</v>
       </c>
+      <c r="D197" t="n">
+        <v>131</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -3989,6 +4593,9 @@
       <c r="C198" s="4" t="n">
         <v>136</v>
       </c>
+      <c r="D198" t="n">
+        <v>167</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
@@ -4004,6 +4611,9 @@
       <c r="C199" s="4" t="n">
         <v>138</v>
       </c>
+      <c r="D199" t="n">
+        <v>169</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
@@ -4019,6 +4629,9 @@
       <c r="C200" s="4" t="n">
         <v>165</v>
       </c>
+      <c r="D200" t="n">
+        <v>210</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
@@ -4034,6 +4647,9 @@
       <c r="C201" s="4" t="n">
         <v>77</v>
       </c>
+      <c r="D201" t="n">
+        <v>94</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
@@ -4049,6 +4665,9 @@
       <c r="C202" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="D202" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
@@ -4064,6 +4683,9 @@
       <c r="C203" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="D203" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
@@ -4079,6 +4701,9 @@
       <c r="C204" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="D204" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
@@ -4094,6 +4719,9 @@
       <c r="C205" s="4" t="n">
         <v>9</v>
       </c>
+      <c r="D205" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
@@ -4109,6 +4737,9 @@
       <c r="C206" s="4" t="n">
         <v>10</v>
       </c>
+      <c r="D206" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
@@ -4124,6 +4755,9 @@
       <c r="C207" s="4" t="n">
         <v>13</v>
       </c>
+      <c r="D207" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
@@ -4139,6 +4773,9 @@
       <c r="C208" s="4" t="n">
         <v>14</v>
       </c>
+      <c r="D208" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
@@ -4154,6 +4791,9 @@
       <c r="C209" s="4" t="n">
         <v>16</v>
       </c>
+      <c r="D209" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
@@ -4169,6 +4809,9 @@
       <c r="C210" s="4" t="n">
         <v>17</v>
       </c>
+      <c r="D210" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
@@ -4184,6 +4827,9 @@
       <c r="C211" s="4" t="n">
         <v>18</v>
       </c>
+      <c r="D211" t="n">
+        <v>97</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
@@ -4199,6 +4845,9 @@
       <c r="C212" s="4" t="n">
         <v>20</v>
       </c>
+      <c r="D212" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
@@ -4214,6 +4863,9 @@
       <c r="C213" s="4" t="n">
         <v>25</v>
       </c>
+      <c r="D213" t="n">
+        <v>119</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
@@ -4229,6 +4881,9 @@
       <c r="C214" s="4" t="n">
         <v>26</v>
       </c>
+      <c r="D214" t="n">
+        <v>121</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
@@ -4244,6 +4899,9 @@
       <c r="C215" s="4" t="n">
         <v>27</v>
       </c>
+      <c r="D215" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
@@ -4259,6 +4917,9 @@
       <c r="C216" s="4" t="n">
         <v>28</v>
       </c>
+      <c r="D216" t="n">
+        <v>141</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
@@ -4274,6 +4935,9 @@
       <c r="C217" s="4" t="n">
         <v>31</v>
       </c>
+      <c r="D217" t="n">
+        <v>163</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
@@ -4289,6 +4953,9 @@
       <c r="C218" s="4" t="n">
         <v>32</v>
       </c>
+      <c r="D218" t="n">
+        <v>173</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
@@ -4304,6 +4971,9 @@
       <c r="C219" s="4" t="n">
         <v>34</v>
       </c>
+      <c r="D219" t="n">
+        <v>176</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
@@ -4319,6 +4989,9 @@
       <c r="C220" s="4" t="n">
         <v>35</v>
       </c>
+      <c r="D220" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
@@ -4334,6 +5007,9 @@
       <c r="C221" s="4" t="n">
         <v>41</v>
       </c>
+      <c r="D221" t="n">
+        <v>196</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
@@ -4349,6 +5025,9 @@
       <c r="C222" s="4" t="n">
         <v>42</v>
       </c>
+      <c r="D222" t="n">
+        <v>197</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
@@ -4364,6 +5043,9 @@
       <c r="C223" s="4" t="n">
         <v>45</v>
       </c>
+      <c r="D223" t="n">
+        <v>202</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
@@ -4379,6 +5061,9 @@
       <c r="C224" s="4" t="n">
         <v>46</v>
       </c>
+      <c r="D224" t="n">
+        <v>216</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
@@ -4394,6 +5079,9 @@
       <c r="C225" s="4" t="n">
         <v>47</v>
       </c>
+      <c r="D225" t="n">
+        <v>224</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
@@ -4409,6 +5097,9 @@
       <c r="C226" s="4" t="n">
         <v>48</v>
       </c>
+      <c r="D226" t="n">
+        <v>240</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
@@ -4424,6 +5115,9 @@
       <c r="C227" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="D227" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
@@ -4439,6 +5133,9 @@
       <c r="C228" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="D228" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
@@ -4454,6 +5151,9 @@
       <c r="C229" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="D229" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
@@ -4469,6 +5169,9 @@
       <c r="C230" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="D230" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
@@ -4484,6 +5187,9 @@
       <c r="C231" s="4" t="n">
         <v>8</v>
       </c>
+      <c r="D231" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
@@ -4499,6 +5205,9 @@
       <c r="C232" s="4" t="n">
         <v>11</v>
       </c>
+      <c r="D232" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
@@ -4514,6 +5223,9 @@
       <c r="C233" s="4" t="n">
         <v>12</v>
       </c>
+      <c r="D233" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
@@ -4529,6 +5241,9 @@
       <c r="C234" s="4" t="n">
         <v>15</v>
       </c>
+      <c r="D234" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
@@ -4544,6 +5259,9 @@
       <c r="C235" s="4" t="n">
         <v>19</v>
       </c>
+      <c r="D235" t="n">
+        <v>98</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
@@ -4559,6 +5277,9 @@
       <c r="C236" s="4" t="n">
         <v>21</v>
       </c>
+      <c r="D236" t="n">
+        <v>109</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
@@ -4574,6 +5295,9 @@
       <c r="C237" s="4" t="n">
         <v>22</v>
       </c>
+      <c r="D237" t="n">
+        <v>112</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
@@ -4589,6 +5313,9 @@
       <c r="C238" s="4" t="n">
         <v>23</v>
       </c>
+      <c r="D238" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
@@ -4604,6 +5331,9 @@
       <c r="C239" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="D239" t="n">
+        <v>115</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
@@ -4619,6 +5349,9 @@
       <c r="C240" s="4" t="n">
         <v>29</v>
       </c>
+      <c r="D240" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
@@ -4634,6 +5367,9 @@
       <c r="C241" s="4" t="n">
         <v>30</v>
       </c>
+      <c r="D241" t="n">
+        <v>160</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
@@ -4649,6 +5385,9 @@
       <c r="C242" s="4" t="n">
         <v>33</v>
       </c>
+      <c r="D242" t="n">
+        <v>174</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
@@ -4664,6 +5403,9 @@
       <c r="C243" s="4" t="n">
         <v>36</v>
       </c>
+      <c r="D243" t="n">
+        <v>184</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
@@ -4679,6 +5421,9 @@
       <c r="C244" s="4" t="n">
         <v>37</v>
       </c>
+      <c r="D244" t="n">
+        <v>185</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
@@ -4694,6 +5439,9 @@
       <c r="C245" s="4" t="n">
         <v>38</v>
       </c>
+      <c r="D245" t="n">
+        <v>191</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
@@ -4709,6 +5457,9 @@
       <c r="C246" s="4" t="n">
         <v>39</v>
       </c>
+      <c r="D246" t="n">
+        <v>194</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
@@ -4724,6 +5475,9 @@
       <c r="C247" s="4" t="n">
         <v>40</v>
       </c>
+      <c r="D247" t="n">
+        <v>195</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
@@ -4739,6 +5493,9 @@
       <c r="C248" s="4" t="n">
         <v>43</v>
       </c>
+      <c r="D248" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
@@ -4754,6 +5511,9 @@
       <c r="C249" s="4" t="n">
         <v>44</v>
       </c>
+      <c r="D249" t="n">
+        <v>201</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
@@ -4768,6 +5528,9 @@
       </c>
       <c r="C250" s="4" t="n">
         <v>49</v>
+      </c>
+      <c r="D250" t="n">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -13356,7 +14119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13373,15 +14136,14 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Table S1. Standard (IID) hard-engine diagnostics (seed 42): engines below 80% Balanced Engine CQR coverage. RMSE, MAE and mean bias (pred − true) in cycles; misses are the share of windows below the lower or above the upper bound; mid-life coverage on windows with 40 &lt; RUL ≤ 80.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>Table S1. Standard (IID) hard-engine diagnostics (seed 42): engines below 80% Balanced Engine CQR coverage. RMSE, MAE and mean bias (pred − true) in cycles; misses are the share of windows below the lower or above the upper bound; mid-life coverage on windows with 40 &lt; RUL ≤ 80. IID engines are identified by FD004 unit number; the number used in the saved prediction files (position among the 49 validation engines) is in the last column.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Engine</t>
+          <t>FD004 unit</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -13422,12 +14184,17 @@
       <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Mid-life cov. (%)</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>IID engine no. in saved files</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>36</v>
+        <v>184</v>
       </c>
       <c r="B4" t="n">
         <v>350</v>
@@ -13453,10 +14220,13 @@
       <c r="I4" t="n">
         <v>30</v>
       </c>
+      <c r="J4" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>37</v>
+        <v>185</v>
       </c>
       <c r="B5" t="n">
         <v>230</v>
@@ -13482,10 +14252,13 @@
       <c r="I5" t="n">
         <v>37.5</v>
       </c>
+      <c r="J5" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>49</v>
+        <v>247</v>
       </c>
       <c r="B6" t="n">
         <v>182</v>
@@ -13510,6 +14283,9 @@
       </c>
       <c r="I6" t="n">
         <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>